<commit_message>
fix dois last pubs
</commit_message>
<xml_diff>
--- a/data/2.full_abstracting/26_02_01_fullabstracting.xlsx
+++ b/data/2.full_abstracting/26_02_01_fullabstracting.xlsx
@@ -409,7 +409,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>10.1016/j.jrp.2026.104705</t>
+          <t>https://doi.org/10.1016/j.jrp.2026.104705</t>
         </is>
       </c>
       <c r="D2">
@@ -484,7 +484,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>10.1177/08902070251409430</t>
+          <t>https://doi.org/10.1177/08902070251409430</t>
         </is>
       </c>
       <c r="D4">
@@ -524,7 +524,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>10.1007/s12187-025-10326-7</t>
+          <t>https://doi.org/10.1007/s12187-025-10326-7</t>
         </is>
       </c>
       <c r="D5">

</xml_diff>